<commit_message>
Add competition scope for SPD and SYS sectionals; enhance judge analytics to support new competition types; implement total activity report across seasons in activity tracker.
</commit_message>
<xml_diff>
--- a/activityAnalysis/US_Champs.xlsx
+++ b/activityAnalysis/US_Champs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rachaelnaphtal/Documents/JudgingAnalysis/activityAnalysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D905D91-A836-A840-B498-1A9462496977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDCDA4B-96C0-5148-92D6-5B6FAEB1E07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15420" yWindow="760" windowWidth="13000" windowHeight="16620" xr2:uid="{891C92EF-756F-2947-96D2-AD9E27690499}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4395" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4409" uniqueCount="528">
   <si>
     <t>Name</t>
   </si>
@@ -1642,6 +1642,9 @@
   <si>
     <t>Ben Wade</t>
   </si>
+  <si>
+    <t>Kitty DeLio-LaForte</t>
+  </si>
 </sst>
 </file>
 
@@ -2734,7 +2737,7 @@
         <v>17</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="R4" s="2"/>
       <c r="S4" s="2" t="s">
@@ -3526,7 +3529,7 @@
         <v>350</v>
       </c>
       <c r="BL7" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="BM7" t="s">
         <v>350</v>
@@ -3972,7 +3975,7 @@
         <v>369</v>
       </c>
       <c r="BF9" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="BG9" t="s">
         <v>350</v>
@@ -4460,7 +4463,7 @@
         <v>350</v>
       </c>
       <c r="BU11" s="8" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="BV11" t="s">
         <v>350</v>
@@ -5781,7 +5784,7 @@
       </c>
       <c r="AV17" s="2"/>
       <c r="AW17" s="2" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="AX17" s="2" t="s">
         <v>9</v>
@@ -5989,7 +5992,7 @@
       </c>
       <c r="AM18" s="2"/>
       <c r="AN18" s="2" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="AO18" s="2" t="s">
         <v>9</v>
@@ -9355,8 +9358,12 @@
         <v>30</v>
       </c>
       <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
+      <c r="P33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q33" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="R33" s="2"/>
       <c r="S33" s="2" t="s">
         <v>56</v>
@@ -9616,7 +9623,7 @@
       </c>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="AF34" s="2" t="s">
         <v>9</v>
@@ -9820,7 +9827,7 @@
       </c>
       <c r="U35" s="2"/>
       <c r="V35" s="2" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="W35" s="2" t="s">
         <v>9</v>
@@ -9902,7 +9909,7 @@
         <v>350</v>
       </c>
       <c r="BF35" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="BG35" t="s">
         <v>350</v>
@@ -11314,7 +11321,7 @@
         <v>369</v>
       </c>
       <c r="CA41" s="8" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="CB41" t="s">
         <v>350</v>
@@ -11633,12 +11640,8 @@
         <v>9</v>
       </c>
       <c r="O43" s="2"/>
-      <c r="P43" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="Q43" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="P43" s="2"/>
+      <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
       <c r="S43" s="2" t="s">
         <v>254</v>
@@ -13620,7 +13623,7 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>334</v>
+        <v>527</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>9</v>
@@ -13851,8 +13854,12 @@
         <v>9</v>
       </c>
       <c r="O53" s="2"/>
-      <c r="P53" s="2"/>
-      <c r="Q53" s="2"/>
+      <c r="P53" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q53" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="R53" s="2"/>
       <c r="S53" s="2" t="s">
         <v>303</v>
@@ -14058,8 +14065,12 @@
         <v>9</v>
       </c>
       <c r="O54" s="2"/>
-      <c r="P54" s="2"/>
-      <c r="Q54" s="2"/>
+      <c r="P54" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q54" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="R54" s="2"/>
       <c r="S54" s="2" t="s">
         <v>62</v>
@@ -14249,8 +14260,12 @@
         <v>9</v>
       </c>
       <c r="O55" s="2"/>
-      <c r="P55" s="2"/>
-      <c r="Q55" s="2"/>
+      <c r="P55" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q55" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="R55" s="2"/>
       <c r="S55" s="2" t="s">
         <v>114</v>
@@ -14408,8 +14423,12 @@
         <v>9</v>
       </c>
       <c r="O56" s="2"/>
-      <c r="P56" s="2"/>
-      <c r="Q56" s="2"/>
+      <c r="P56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q56" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="R56" s="2"/>
       <c r="S56" s="2" t="s">
         <v>105</v>
@@ -14563,8 +14582,12 @@
         <v>9</v>
       </c>
       <c r="O57" s="2"/>
-      <c r="P57" s="2"/>
-      <c r="Q57" s="2"/>
+      <c r="P57" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q57" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="R57" s="2"/>
       <c r="S57" s="2" t="s">
         <v>111</v>
@@ -14704,8 +14727,12 @@
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
-      <c r="P58" s="2"/>
-      <c r="Q58" s="2"/>
+      <c r="P58" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q58" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="R58" s="2"/>
       <c r="S58" s="2" t="s">
         <v>319</v>
@@ -14845,8 +14872,12 @@
         <v>131</v>
       </c>
       <c r="O59" s="2"/>
-      <c r="P59" s="2"/>
-      <c r="Q59" s="2"/>
+      <c r="P59" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q59" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="R59" s="2"/>
       <c r="S59" s="2" t="s">
         <v>157</v>
@@ -14975,12 +15006,8 @@
         <v>9</v>
       </c>
       <c r="L60" s="2"/>
-      <c r="M60" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="N60" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="M60" s="2"/>
+      <c r="N60" s="2"/>
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
       <c r="Q60" s="2"/>
@@ -15372,8 +15399,12 @@
         <v>9</v>
       </c>
       <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
-      <c r="N63" s="2"/>
+      <c r="M63" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N63" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
       <c r="Q63" s="2"/>

</xml_diff>